<commit_message>
feat: add loop to method
</commit_message>
<xml_diff>
--- a/docs/Lab03/Lab03_WBT_TCs_Form.xlsx
+++ b/docs/Lab03/Lab03_WBT_TCs_Form.xlsx
@@ -118,7 +118,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">cautarea filmelor care au un anumit regizor (sau parti din numele regizorului).</t>
+      <t xml:space="preserve">Actualizarea unui produs (validarea modificarilor aduse)</t>
     </r>
   </si>
   <si>
@@ -194,13 +194,13 @@
     <t xml:space="preserve">F02_P01</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (F) – 7(F) – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(F) – 8(F) – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P02</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (F) – 7(F) – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(F) – 8(F) – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p1</t>
@@ -209,31 +209,31 @@
     <t xml:space="preserve">F02_P03</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(T) – 6 – 7(F) – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(T) – 7 – 8(F) – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P04</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (T) – 6 – 7(F) – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(T) – 7 – 8(F) – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P05</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (F) – 7(T) – 8 – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(F) – 8(T) – 9 – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P06</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (F) – 7(F) – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(F) – 8(F) – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P07</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(T) – 6 – 7(F) – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(T) – 7  – 8(F) – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p2</t>
@@ -242,25 +242,25 @@
     <t xml:space="preserve">F02_P08</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (T) – 6 – 7(F) – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(T) – 7 – 8(F) – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P09</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (F) – 7(T) – 8 – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(F) – 8(T) – 9 – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P10</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (F) – 7(F) – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(F) – 8(F) – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P11</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(T) – 6 – 7(T) – 8 – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(T) – 7 – 8(T) – 9 – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p3</t>
@@ -269,13 +269,13 @@
     <t xml:space="preserve">F02_P12</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(T) – 6 – 7(F) – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(T) – 7 – 8(F) – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P13</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (T) – 6 – 7(T) – 8 – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(T) – 7 – 8(T) – 9 – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p4</t>
@@ -284,13 +284,13 @@
     <t xml:space="preserve">F02_P14</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (T) – 6 – 7(F) – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(T) – 7 – 8(F) – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P15</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (F) – 7(T) – 8 – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(F) – 8(T) – 9 – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p5</t>
@@ -299,7 +299,7 @@
     <t xml:space="preserve">F02_P16</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(T) – 6 – 7(T) – 8 – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(T) – 7  – 8(T) – 9 – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p7</t>
@@ -308,13 +308,13 @@
     <t xml:space="preserve">F02_P17</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(T) – 6 – 7(F) – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(T) – 7  – 8(F) – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P18</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (T) – 6 – 7(T) – 8 – 9(F) – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(T) – 7 – 8(T) – 9 – 10(F) – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p8</t>
@@ -323,13 +323,13 @@
     <t xml:space="preserve">F02_P19</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (T) – 6 – 7(F) – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(T) – 7 – 8(F) – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">F02_P20</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (F) – 7(T) – 8 – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(F) – 8(T) – 9 – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p9</t>
@@ -338,7 +338,7 @@
     <t xml:space="preserve">F02_P21</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(T) – 6 – 7(T) – 8 – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(T) – 7 – 8(T) – 9 – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p11</t>
@@ -347,7 +347,7 @@
     <t xml:space="preserve">F02_P22</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(F) – 4(F) – 5 (T) – 6 – 7(T) – 8 – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(F) – 5(F) – 6(T) – 7 – 8(T) – 9 – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p13</t>
@@ -356,7 +356,7 @@
     <t xml:space="preserve">F02_P23</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(T) – 6 – 7(T) – 8 – 9(T) – 10 – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(T) – 7  – 8(T) – 9 – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p16</t>
@@ -365,7 +365,7 @@
     <t xml:space="preserve">F02_P24</t>
   </si>
   <si>
-    <t xml:space="preserve">1 – 2(T) – 3 – 4(F) – 5 (T) – 6 – 7(T) – 8 – 9(T) - 10 – 11</t>
+    <t xml:space="preserve">1 – 2(T) – 3 – 4 – 2(F) – 5(F) – 6(T) – 7 – 8(T) – 9 – 10(T) – 11 – 12</t>
   </si>
   <si>
     <t xml:space="preserve">p18</t>
@@ -1188,292 +1188,296 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="9" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="8" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="8" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="10" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="10" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="11" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="11" borderId="21" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="21" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="23" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="23" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="23" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="12" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="12" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="12" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="12" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="11" borderId="23" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="23" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="12" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="12" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="12" borderId="24" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="24" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1553,20 +1557,20 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>3600</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>701640</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>-360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>701280</xdr:colOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>11880</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>63720</xdr:rowOff>
+      <xdr:rowOff>151200</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="1" name="Image 1"/>
+        <xdr:cNvPr id="1" name="Image 3"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1575,8 +1579,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="712440" y="1293840"/>
-          <a:ext cx="4332240" cy="2959560"/>
+          <a:off x="701640" y="1293840"/>
+          <a:ext cx="4362480" cy="3047040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1592,19 +1596,19 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>696960</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>170640</xdr:rowOff>
+      <xdr:colOff>472680</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>-360</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>15</xdr:col>
-      <xdr:colOff>28080</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>180720</xdr:rowOff>
+      <xdr:colOff>266040</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>1440</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Image 2"/>
+        <xdr:cNvPr id="2" name="Image 1"/>
         <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
@@ -1613,8 +1617,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5749200" y="1283760"/>
-          <a:ext cx="5000400" cy="10144800"/>
+          <a:off x="5524920" y="1293840"/>
+          <a:ext cx="5462640" cy="8688600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1814,130 +1818,130 @@
   <dimension ref="B1:P20"/>
   <sheetFormatPr defaultColWidth="8.859375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="15.93"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="39.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="21.85"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="15.93"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="39.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="21.85"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1"/>
-      <c r="D1" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="N4" s="5" t="s">
+      <c r="N4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="N5" s="6" t="s">
+      <c r="N5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="O5" s="6"/>
-      <c r="P5" s="6"/>
+      <c r="O5" s="7"/>
+      <c r="P5" s="7"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="N6" s="7"/>
-      <c r="O6" s="7" t="s">
+      <c r="N6" s="8"/>
+      <c r="O6" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="P6" s="7" t="s">
+      <c r="P6" s="8" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="N7" s="7" t="s">
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="N7" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="O7" s="7" t="s">
+      <c r="O7" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="P7" s="7" t="n">
+      <c r="P7" s="8" t="n">
         <v>234</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="4"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="N8" s="7" t="s">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="N8" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="O8" s="7" t="s">
+      <c r="O8" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="P8" s="7" t="n">
+      <c r="P8" s="8" t="n">
         <v>234</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="N9" s="7" t="s">
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="N9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="O9" s="7" t="s">
+      <c r="O9" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="P9" s="7" t="n">
+      <c r="P9" s="8" t="n">
         <v>234</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="4"/>
+      <c r="B19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4"/>
+      <c r="B20" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1962,635 +1966,635 @@
   <dimension ref="B1:U43"/>
   <sheetFormatPr defaultColWidth="8.859375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="10.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="14.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="19.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="17.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="10.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="14.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="19.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="17.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1"/>
-      <c r="D1" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
+      <c r="J3" s="10"/>
+      <c r="K3" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="I6" s="11" t="s">
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="I6" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="Q6" s="11" t="s">
+      <c r="J6" s="12"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="12"/>
+      <c r="M6" s="12"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+      <c r="Q6" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="11"/>
-      <c r="S6" s="11"/>
-      <c r="T6" s="11"/>
+      <c r="R6" s="12"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="12"/>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-      <c r="I8" s="1" t="s">
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
+      <c r="I8" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Q8" s="14" t="s">
+      <c r="Q8" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
-      <c r="T8" s="15" t="n">
+      <c r="R8" s="15"/>
+      <c r="S8" s="15"/>
+      <c r="T8" s="16" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="16"/>
-      <c r="G9" s="16"/>
-      <c r="I9" s="17"/>
-      <c r="Q9" s="14" t="s">
+      <c r="C9" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="I9" s="18"/>
+      <c r="Q9" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="R9" s="14"/>
-      <c r="S9" s="14"/>
-      <c r="T9" s="15" t="s">
+      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
+      <c r="T9" s="16" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="16"/>
-      <c r="G10" s="16"/>
-      <c r="I10" s="18" t="s">
+      <c r="C10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="I10" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
-      <c r="Q10" s="14" t="s">
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="Q10" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="R10" s="14" t="s">
+      <c r="R10" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="S10" s="14"/>
-      <c r="T10" s="15" t="s">
+      <c r="S10" s="15"/>
+      <c r="T10" s="16" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="16"/>
-      <c r="G11" s="16"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
-      <c r="N11" s="18"/>
-      <c r="O11" s="18"/>
+      <c r="C11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="16"/>
-      <c r="G12" s="16"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
+      <c r="C12" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="16"/>
-      <c r="G13" s="16"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="18"/>
-      <c r="N13" s="18"/>
-      <c r="O13" s="18"/>
-      <c r="Q13" s="11" t="s">
+      <c r="C13" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="19"/>
+      <c r="L13" s="19"/>
+      <c r="M13" s="19"/>
+      <c r="N13" s="19"/>
+      <c r="O13" s="19"/>
+      <c r="Q13" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="R13" s="11"/>
-      <c r="S13" s="11"/>
-      <c r="T13" s="11"/>
+      <c r="R13" s="12"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="12"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="16"/>
-      <c r="G14" s="16"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="18"/>
+      <c r="C14" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I15" s="18"/>
-      <c r="J15" s="18"/>
-      <c r="K15" s="18"/>
-      <c r="L15" s="18"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="18"/>
-      <c r="O15" s="18"/>
-      <c r="Q15" s="12" t="s">
+      <c r="I15" s="19"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="19"/>
+      <c r="L15" s="19"/>
+      <c r="M15" s="19"/>
+      <c r="N15" s="19"/>
+      <c r="O15" s="19"/>
+      <c r="Q15" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="R15" s="12" t="s">
+      <c r="R15" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="S15" s="12"/>
-      <c r="T15" s="12"/>
-      <c r="U15" s="0" t="s">
+      <c r="S15" s="13"/>
+      <c r="T15" s="13"/>
+      <c r="U15" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18"/>
-      <c r="N16" s="18"/>
-      <c r="O16" s="18"/>
-      <c r="Q16" s="6" t="s">
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
+      <c r="L16" s="19"/>
+      <c r="M16" s="19"/>
+      <c r="N16" s="19"/>
+      <c r="O16" s="19"/>
+      <c r="Q16" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="R16" s="19" t="s">
+      <c r="R16" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="S16" s="19"/>
-      <c r="T16" s="19"/>
+      <c r="S16" s="20"/>
+      <c r="T16" s="20"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
-      <c r="N17" s="18"/>
-      <c r="O17" s="18"/>
-      <c r="Q17" s="6" t="s">
+      <c r="I17" s="19"/>
+      <c r="J17" s="19"/>
+      <c r="K17" s="19"/>
+      <c r="L17" s="19"/>
+      <c r="M17" s="19"/>
+      <c r="N17" s="19"/>
+      <c r="O17" s="19"/>
+      <c r="Q17" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="R17" s="19" t="s">
+      <c r="R17" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="S17" s="19"/>
-      <c r="T17" s="19"/>
-      <c r="U17" s="0" t="s">
+      <c r="S17" s="20"/>
+      <c r="T17" s="20"/>
+      <c r="U17" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
-      <c r="Q18" s="6" t="s">
+      <c r="I18" s="19"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="19"/>
+      <c r="L18" s="19"/>
+      <c r="M18" s="19"/>
+      <c r="N18" s="19"/>
+      <c r="O18" s="19"/>
+      <c r="Q18" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="R18" s="19" t="s">
+      <c r="R18" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="S18" s="19"/>
-      <c r="T18" s="19"/>
-      <c r="U18" s="0" t="s">
+      <c r="S18" s="20"/>
+      <c r="T18" s="20"/>
+      <c r="U18" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-      <c r="Q19" s="6" t="s">
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19"/>
+      <c r="Q19" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="R19" s="19" t="s">
+      <c r="R19" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="S19" s="19"/>
-      <c r="T19" s="19"/>
-      <c r="U19" s="0" t="s">
+      <c r="S19" s="20"/>
+      <c r="T19" s="20"/>
+      <c r="U19" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I20" s="18"/>
-      <c r="J20" s="18"/>
-      <c r="K20" s="18"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="18"/>
-      <c r="N20" s="18"/>
-      <c r="O20" s="18"/>
-      <c r="Q20" s="6" t="s">
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="19"/>
+      <c r="Q20" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="R20" s="19" t="s">
+      <c r="R20" s="20" t="s">
         <v>52</v>
       </c>
-      <c r="S20" s="19"/>
-      <c r="T20" s="19"/>
-      <c r="U20" s="0" t="s">
+      <c r="S20" s="20"/>
+      <c r="T20" s="20"/>
+      <c r="U20" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="18"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="18"/>
-      <c r="N21" s="18"/>
-      <c r="O21" s="18"/>
-      <c r="Q21" s="6" t="s">
+      <c r="I21" s="19"/>
+      <c r="J21" s="19"/>
+      <c r="K21" s="19"/>
+      <c r="L21" s="19"/>
+      <c r="M21" s="19"/>
+      <c r="N21" s="19"/>
+      <c r="O21" s="19"/>
+      <c r="Q21" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="R21" s="19" t="s">
+      <c r="R21" s="20" t="s">
         <v>54</v>
       </c>
-      <c r="S21" s="19"/>
-      <c r="T21" s="19"/>
-      <c r="U21" s="0" t="s">
+      <c r="S21" s="20"/>
+      <c r="T21" s="20"/>
+      <c r="U21" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I22" s="18"/>
-      <c r="J22" s="18"/>
-      <c r="K22" s="18"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="18"/>
-      <c r="N22" s="18"/>
-      <c r="O22" s="18"/>
-      <c r="Q22" s="6" t="s">
+      <c r="I22" s="19"/>
+      <c r="J22" s="19"/>
+      <c r="K22" s="19"/>
+      <c r="L22" s="19"/>
+      <c r="M22" s="19"/>
+      <c r="N22" s="19"/>
+      <c r="O22" s="19"/>
+      <c r="Q22" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="R22" s="19" t="s">
+      <c r="R22" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="S22" s="19"/>
-      <c r="T22" s="19"/>
-      <c r="U22" s="0" t="s">
+      <c r="S22" s="20"/>
+      <c r="T22" s="20"/>
+      <c r="U22" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="18"/>
-      <c r="N23" s="18"/>
-      <c r="O23" s="18"/>
-      <c r="Q23" s="6" t="s">
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+      <c r="O23" s="19"/>
+      <c r="Q23" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="R23" s="19" t="s">
+      <c r="R23" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="S23" s="19"/>
-      <c r="T23" s="19"/>
-      <c r="U23" s="0" t="s">
+      <c r="S23" s="20"/>
+      <c r="T23" s="20"/>
+      <c r="U23" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="18"/>
-      <c r="N24" s="18"/>
-      <c r="O24" s="18"/>
-      <c r="Q24" s="6" t="s">
+      <c r="I24" s="19"/>
+      <c r="J24" s="19"/>
+      <c r="K24" s="19"/>
+      <c r="L24" s="19"/>
+      <c r="M24" s="19"/>
+      <c r="N24" s="19"/>
+      <c r="O24" s="19"/>
+      <c r="Q24" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="R24" s="19" t="s">
+      <c r="R24" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="S24" s="19"/>
-      <c r="T24" s="19"/>
-      <c r="U24" s="0" t="s">
+      <c r="S24" s="20"/>
+      <c r="T24" s="20"/>
+      <c r="U24" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q25" s="6" t="s">
+      <c r="Q25" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="R25" s="19" t="s">
+      <c r="R25" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="S25" s="19"/>
-      <c r="T25" s="19"/>
-      <c r="U25" s="0" t="s">
+      <c r="S25" s="20"/>
+      <c r="T25" s="20"/>
+      <c r="U25" s="1" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q26" s="6" t="s">
+      <c r="Q26" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="R26" s="19" t="s">
+      <c r="R26" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="S26" s="19"/>
-      <c r="T26" s="19"/>
-      <c r="U26" s="0" t="s">
+      <c r="S26" s="20"/>
+      <c r="T26" s="20"/>
+      <c r="U26" s="1" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q27" s="6" t="s">
+      <c r="Q27" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="R27" s="19" t="s">
+      <c r="R27" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="S27" s="19"/>
-      <c r="T27" s="19"/>
-      <c r="U27" s="0" t="s">
+      <c r="S27" s="20"/>
+      <c r="T27" s="20"/>
+      <c r="U27" s="1" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q28" s="6" t="s">
+      <c r="Q28" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="R28" s="19" t="s">
+      <c r="R28" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="S28" s="19"/>
-      <c r="T28" s="19"/>
-      <c r="U28" s="0" t="s">
+      <c r="S28" s="20"/>
+      <c r="T28" s="20"/>
+      <c r="U28" s="1" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q29" s="6" t="s">
+      <c r="Q29" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="R29" s="19" t="s">
+      <c r="R29" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="S29" s="19"/>
-      <c r="T29" s="19"/>
-      <c r="U29" s="0" t="s">
+      <c r="S29" s="20"/>
+      <c r="T29" s="20"/>
+      <c r="U29" s="1" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q30" s="6" t="s">
+      <c r="Q30" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="R30" s="19" t="s">
+      <c r="R30" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="S30" s="19"/>
-      <c r="T30" s="19"/>
-      <c r="U30" s="0" t="s">
+      <c r="S30" s="20"/>
+      <c r="T30" s="20"/>
+      <c r="U30" s="1" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q31" s="6" t="s">
+      <c r="Q31" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="R31" s="19" t="s">
+      <c r="R31" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="S31" s="19"/>
-      <c r="T31" s="19"/>
-      <c r="U31" s="0" t="s">
+      <c r="S31" s="20"/>
+      <c r="T31" s="20"/>
+      <c r="U31" s="1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q32" s="6" t="s">
+      <c r="Q32" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="R32" s="19" t="s">
+      <c r="R32" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="S32" s="19"/>
-      <c r="T32" s="19"/>
-      <c r="U32" s="0" t="s">
+      <c r="S32" s="20"/>
+      <c r="T32" s="20"/>
+      <c r="U32" s="1" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q33" s="6" t="s">
+      <c r="Q33" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="R33" s="19" t="s">
+      <c r="R33" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="S33" s="19"/>
-      <c r="T33" s="19"/>
-      <c r="U33" s="0" t="s">
+      <c r="S33" s="20"/>
+      <c r="T33" s="20"/>
+      <c r="U33" s="1" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q34" s="6" t="s">
+      <c r="Q34" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="R34" s="19" t="s">
+      <c r="R34" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="S34" s="19"/>
-      <c r="T34" s="19"/>
-      <c r="U34" s="0" t="s">
+      <c r="S34" s="20"/>
+      <c r="T34" s="20"/>
+      <c r="U34" s="1" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q35" s="6" t="s">
+      <c r="Q35" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="R35" s="19" t="s">
+      <c r="R35" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="S35" s="19"/>
-      <c r="T35" s="19"/>
-      <c r="U35" s="0" t="s">
+      <c r="S35" s="20"/>
+      <c r="T35" s="20"/>
+      <c r="U35" s="1" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q36" s="6" t="s">
+      <c r="Q36" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="R36" s="19" t="s">
+      <c r="R36" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="S36" s="19"/>
-      <c r="T36" s="19"/>
-      <c r="U36" s="0" t="s">
+      <c r="S36" s="20"/>
+      <c r="T36" s="20"/>
+      <c r="U36" s="1" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q37" s="6" t="s">
+      <c r="Q37" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="R37" s="19" t="s">
+      <c r="R37" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="S37" s="19"/>
-      <c r="T37" s="19"/>
-      <c r="U37" s="0" t="s">
+      <c r="S37" s="20"/>
+      <c r="T37" s="20"/>
+      <c r="U37" s="1" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q38" s="6" t="s">
+      <c r="Q38" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="R38" s="19" t="s">
+      <c r="R38" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="S38" s="19"/>
-      <c r="T38" s="19"/>
-      <c r="U38" s="0" t="s">
+      <c r="S38" s="20"/>
+      <c r="T38" s="20"/>
+      <c r="U38" s="1" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q39" s="6" t="s">
+      <c r="Q39" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="R39" s="19" t="s">
+      <c r="R39" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="S39" s="19"/>
-      <c r="T39" s="19"/>
-      <c r="U39" s="0" t="s">
+      <c r="S39" s="20"/>
+      <c r="T39" s="20"/>
+      <c r="U39" s="1" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q40" s="6"/>
-      <c r="R40" s="19"/>
-      <c r="S40" s="19"/>
-      <c r="T40" s="19"/>
+      <c r="Q40" s="7"/>
+      <c r="R40" s="20"/>
+      <c r="S40" s="20"/>
+      <c r="T40" s="20"/>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q41" s="6"/>
-      <c r="R41" s="19"/>
-      <c r="S41" s="19"/>
-      <c r="T41" s="19"/>
+      <c r="Q41" s="7"/>
+      <c r="R41" s="20"/>
+      <c r="S41" s="20"/>
+      <c r="T41" s="20"/>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q42" s="6"/>
-      <c r="R42" s="19"/>
-      <c r="S42" s="19"/>
-      <c r="T42" s="19"/>
+      <c r="Q42" s="7"/>
+      <c r="R42" s="20"/>
+      <c r="S42" s="20"/>
+      <c r="T42" s="20"/>
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="Q43" s="6"/>
-      <c r="R43" s="19"/>
-      <c r="S43" s="19"/>
-      <c r="T43" s="19"/>
+      <c r="Q43" s="7"/>
+      <c r="R43" s="20"/>
+      <c r="S43" s="20"/>
+      <c r="T43" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="46">
@@ -2661,437 +2665,437 @@
   <dimension ref="B1:AB16"/>
   <sheetFormatPr defaultColWidth="8.859375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="18.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="19.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="8.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="14.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="6.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="6.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="11.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="9.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="22" style="0" width="2.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="3.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="0" width="2.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="0" width="4.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="0" width="5.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="18.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="19.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="8.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="11.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="11.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="14.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="6.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="6.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="9.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="22" style="1" width="2.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="1" width="3.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="26" style="1" width="2.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="27" min="27" style="1" width="4.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="28" min="28" style="1" width="5.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1"/>
-      <c r="D1" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="20"/>
+      <c r="B5" s="21"/>
     </row>
     <row r="6" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="E6" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="21"/>
-      <c r="J6" s="21"/>
-      <c r="K6" s="21"/>
-      <c r="L6" s="21"/>
-      <c r="M6" s="21"/>
-      <c r="N6" s="21"/>
-      <c r="O6" s="21"/>
-      <c r="P6" s="21"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="21"/>
-      <c r="U6" s="21"/>
-      <c r="V6" s="21"/>
-      <c r="W6" s="21"/>
-      <c r="X6" s="21"/>
-      <c r="Y6" s="21"/>
-      <c r="Z6" s="21"/>
-      <c r="AA6" s="21"/>
-      <c r="AB6" s="21"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
+      <c r="O6" s="22"/>
+      <c r="P6" s="22"/>
+      <c r="Q6" s="22"/>
+      <c r="R6" s="22"/>
+      <c r="S6" s="22"/>
+      <c r="T6" s="22"/>
+      <c r="U6" s="22"/>
+      <c r="V6" s="22"/>
+      <c r="W6" s="22"/>
+      <c r="X6" s="22"/>
+      <c r="Y6" s="22"/>
+      <c r="Z6" s="22"/>
+      <c r="AA6" s="22"/>
+      <c r="AB6" s="22"/>
     </row>
     <row r="7" customFormat="false" ht="17.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="22" t="s">
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23" t="s">
         <v>106</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="F7" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="23"/>
-      <c r="L7" s="23"/>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="24" t="s">
+      <c r="G7" s="24"/>
+      <c r="H7" s="24"/>
+      <c r="I7" s="24"/>
+      <c r="J7" s="24"/>
+      <c r="K7" s="24"/>
+      <c r="L7" s="24"/>
+      <c r="M7" s="24"/>
+      <c r="N7" s="24"/>
+      <c r="O7" s="24"/>
+      <c r="P7" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="Q7" s="24"/>
-      <c r="R7" s="24"/>
-      <c r="S7" s="24"/>
-      <c r="T7" s="24"/>
-      <c r="U7" s="24"/>
-      <c r="V7" s="25" t="s">
+      <c r="Q7" s="25"/>
+      <c r="R7" s="25"/>
+      <c r="S7" s="25"/>
+      <c r="T7" s="25"/>
+      <c r="U7" s="25"/>
+      <c r="V7" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="W7" s="25"/>
-      <c r="X7" s="25"/>
-      <c r="Y7" s="25"/>
-      <c r="Z7" s="25"/>
-      <c r="AA7" s="25"/>
-      <c r="AB7" s="25"/>
+      <c r="W7" s="26"/>
+      <c r="X7" s="26"/>
+      <c r="Y7" s="26"/>
+      <c r="Z7" s="26"/>
+      <c r="AA7" s="26"/>
+      <c r="AB7" s="26"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="21"/>
-      <c r="C8" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="26" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="22"/>
-      <c r="F8" s="23" t="s">
+      <c r="B8" s="22"/>
+      <c r="C8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="23"/>
+      <c r="F8" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23" t="s">
+      <c r="G8" s="24"/>
+      <c r="H8" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23" t="s">
+      <c r="I8" s="24"/>
+      <c r="J8" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23" t="s">
+      <c r="K8" s="24"/>
+      <c r="L8" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="O8" s="23"/>
-      <c r="P8" s="24" t="s">
+      <c r="O8" s="24"/>
+      <c r="P8" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="Q8" s="24" t="s">
+      <c r="Q8" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="R8" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="S8" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="T8" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="U8" s="24" t="s">
+      <c r="R8" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="T8" s="25" t="s">
+        <v>27</v>
+      </c>
+      <c r="U8" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="V8" s="25" t="n">
+      <c r="V8" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="W8" s="25" t="n">
+      <c r="W8" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="X8" s="25" t="n">
+      <c r="X8" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Y8" s="25" t="s">
+      <c r="Y8" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="Z8" s="25" t="s">
+      <c r="Z8" s="26" t="s">
         <v>116</v>
       </c>
-      <c r="AA8" s="25" t="s">
+      <c r="AA8" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="AB8" s="25" t="s">
+      <c r="AB8" s="26" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="21"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="23" t="s">
+      <c r="B9" s="22"/>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="H9" s="23" t="s">
+      <c r="H9" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="I9" s="23" t="s">
+      <c r="I9" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="J9" s="23" t="s">
+      <c r="J9" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="K9" s="23" t="s">
+      <c r="K9" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="M9" s="23" t="s">
+      <c r="M9" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="N9" s="23" t="s">
+      <c r="N9" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="O9" s="23" t="s">
+      <c r="O9" s="24" t="s">
         <v>120</v>
       </c>
-      <c r="P9" s="24"/>
-      <c r="Q9" s="24"/>
-      <c r="R9" s="24"/>
-      <c r="S9" s="24"/>
-      <c r="T9" s="24"/>
-      <c r="U9" s="24"/>
-      <c r="V9" s="25"/>
-      <c r="W9" s="25"/>
-      <c r="X9" s="25"/>
-      <c r="Y9" s="25"/>
-      <c r="Z9" s="25"/>
-      <c r="AA9" s="25"/>
-      <c r="AB9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="25"/>
+      <c r="R9" s="25"/>
+      <c r="S9" s="25"/>
+      <c r="T9" s="25"/>
+      <c r="U9" s="25"/>
+      <c r="V9" s="26"/>
+      <c r="W9" s="26"/>
+      <c r="X9" s="26"/>
+      <c r="Y9" s="26"/>
+      <c r="Z9" s="26"/>
+      <c r="AA9" s="26"/>
+      <c r="AB9" s="26"/>
     </row>
     <row r="10" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="28" t="s">
         <v>121</v>
       </c>
-      <c r="C10" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="29" t="s">
+      <c r="C10" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="F10" s="30"/>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-      <c r="I10" s="30"/>
-      <c r="J10" s="30"/>
-      <c r="K10" s="30"/>
-      <c r="L10" s="30"/>
-      <c r="M10" s="30"/>
-      <c r="N10" s="30"/>
-      <c r="O10" s="30"/>
-      <c r="P10" s="31"/>
-      <c r="Q10" s="31"/>
-      <c r="R10" s="31"/>
-      <c r="S10" s="31"/>
-      <c r="T10" s="31"/>
-      <c r="U10" s="31"/>
-      <c r="V10" s="32"/>
-      <c r="W10" s="32"/>
-      <c r="X10" s="32"/>
-      <c r="Y10" s="32"/>
-      <c r="Z10" s="32"/>
-      <c r="AA10" s="32"/>
-      <c r="AB10" s="32"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="31"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
+      <c r="O10" s="31"/>
+      <c r="P10" s="32"/>
+      <c r="Q10" s="32"/>
+      <c r="R10" s="32"/>
+      <c r="S10" s="32"/>
+      <c r="T10" s="32"/>
+      <c r="U10" s="32"/>
+      <c r="V10" s="33"/>
+      <c r="W10" s="33"/>
+      <c r="X10" s="33"/>
+      <c r="Y10" s="33"/>
+      <c r="Z10" s="33"/>
+      <c r="AA10" s="33"/>
+      <c r="AB10" s="33"/>
     </row>
     <row r="11" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="28" t="s">
         <v>123</v>
       </c>
-      <c r="C11" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" s="28" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="29"/>
-      <c r="F11" s="30"/>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-      <c r="I11" s="30"/>
-      <c r="J11" s="30"/>
-      <c r="K11" s="30"/>
-      <c r="L11" s="30"/>
-      <c r="M11" s="30"/>
-      <c r="N11" s="30"/>
-      <c r="O11" s="30"/>
-      <c r="P11" s="31"/>
-      <c r="Q11" s="31"/>
-      <c r="R11" s="31"/>
-      <c r="S11" s="31"/>
-      <c r="T11" s="31"/>
-      <c r="U11" s="31"/>
-      <c r="V11" s="32"/>
-      <c r="W11" s="32"/>
-      <c r="X11" s="32"/>
-      <c r="Y11" s="32"/>
-      <c r="Z11" s="32"/>
-      <c r="AA11" s="32"/>
-      <c r="AB11" s="32"/>
+      <c r="C11" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="29" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="30"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
+      <c r="O11" s="31"/>
+      <c r="P11" s="32"/>
+      <c r="Q11" s="32"/>
+      <c r="R11" s="32"/>
+      <c r="S11" s="32"/>
+      <c r="T11" s="32"/>
+      <c r="U11" s="32"/>
+      <c r="V11" s="33"/>
+      <c r="W11" s="33"/>
+      <c r="X11" s="33"/>
+      <c r="Y11" s="33"/>
+      <c r="Z11" s="33"/>
+      <c r="AA11" s="33"/>
+      <c r="AB11" s="33"/>
     </row>
     <row r="12" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="33"/>
-      <c r="D12" s="34"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="30"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-      <c r="I12" s="30"/>
-      <c r="J12" s="30"/>
-      <c r="K12" s="30"/>
-      <c r="L12" s="30"/>
-      <c r="M12" s="30"/>
-      <c r="N12" s="30"/>
-      <c r="O12" s="30"/>
-      <c r="P12" s="31"/>
-      <c r="Q12" s="31"/>
-      <c r="R12" s="31"/>
-      <c r="S12" s="31"/>
-      <c r="T12" s="31"/>
-      <c r="U12" s="31"/>
-      <c r="V12" s="32"/>
-      <c r="W12" s="32"/>
-      <c r="X12" s="32"/>
-      <c r="Y12" s="32"/>
-      <c r="Z12" s="32"/>
-      <c r="AA12" s="32"/>
-      <c r="AB12" s="32"/>
+      <c r="B12" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="34"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="30"/>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="31"/>
+      <c r="O12" s="31"/>
+      <c r="P12" s="32"/>
+      <c r="Q12" s="32"/>
+      <c r="R12" s="32"/>
+      <c r="S12" s="32"/>
+      <c r="T12" s="32"/>
+      <c r="U12" s="32"/>
+      <c r="V12" s="33"/>
+      <c r="W12" s="33"/>
+      <c r="X12" s="33"/>
+      <c r="Y12" s="33"/>
+      <c r="Z12" s="33"/>
+      <c r="AA12" s="33"/>
+      <c r="AB12" s="33"/>
     </row>
     <row r="13" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C13" s="27"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="29"/>
-      <c r="F13" s="30"/>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
-      <c r="K13" s="30"/>
-      <c r="L13" s="30"/>
-      <c r="M13" s="30"/>
-      <c r="N13" s="30"/>
-      <c r="O13" s="30"/>
-      <c r="P13" s="31"/>
-      <c r="Q13" s="31"/>
-      <c r="R13" s="31"/>
-      <c r="S13" s="31"/>
-      <c r="T13" s="31"/>
-      <c r="U13" s="31"/>
-      <c r="V13" s="32"/>
-      <c r="W13" s="32"/>
-      <c r="X13" s="32"/>
-      <c r="Y13" s="32"/>
-      <c r="Z13" s="32"/>
-      <c r="AA13" s="32"/>
-      <c r="AB13" s="32"/>
+      <c r="B13" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="28"/>
+      <c r="D13" s="29"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="31"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
+      <c r="J13" s="31"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
+      <c r="O13" s="31"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="32"/>
+      <c r="R13" s="32"/>
+      <c r="S13" s="32"/>
+      <c r="T13" s="32"/>
+      <c r="U13" s="32"/>
+      <c r="V13" s="33"/>
+      <c r="W13" s="33"/>
+      <c r="X13" s="33"/>
+      <c r="Y13" s="33"/>
+      <c r="Z13" s="33"/>
+      <c r="AA13" s="33"/>
+      <c r="AB13" s="33"/>
     </row>
     <row r="14" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" s="27"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="29"/>
-      <c r="F14" s="30"/>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-      <c r="I14" s="30"/>
-      <c r="J14" s="30"/>
-      <c r="K14" s="30"/>
-      <c r="L14" s="30"/>
-      <c r="M14" s="30"/>
-      <c r="N14" s="30"/>
-      <c r="O14" s="30"/>
-      <c r="P14" s="31"/>
-      <c r="Q14" s="31"/>
-      <c r="R14" s="31"/>
-      <c r="S14" s="31"/>
-      <c r="T14" s="31"/>
-      <c r="U14" s="31"/>
-      <c r="V14" s="32"/>
-      <c r="W14" s="32"/>
-      <c r="X14" s="32"/>
-      <c r="Y14" s="32"/>
-      <c r="Z14" s="32"/>
-      <c r="AA14" s="32"/>
-      <c r="AB14" s="32"/>
+      <c r="B14" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="28"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="31"/>
+      <c r="N14" s="31"/>
+      <c r="O14" s="31"/>
+      <c r="P14" s="32"/>
+      <c r="Q14" s="32"/>
+      <c r="R14" s="32"/>
+      <c r="S14" s="32"/>
+      <c r="T14" s="32"/>
+      <c r="U14" s="32"/>
+      <c r="V14" s="33"/>
+      <c r="W14" s="33"/>
+      <c r="X14" s="33"/>
+      <c r="Y14" s="33"/>
+      <c r="Z14" s="33"/>
+      <c r="AA14" s="33"/>
+      <c r="AB14" s="33"/>
     </row>
     <row r="15" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="27" t="s">
-        <v>27</v>
-      </c>
-      <c r="C15" s="27"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="29"/>
-      <c r="F15" s="30"/>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="30"/>
-      <c r="K15" s="30"/>
-      <c r="L15" s="30"/>
-      <c r="M15" s="30"/>
-      <c r="N15" s="30"/>
-      <c r="O15" s="30"/>
-      <c r="P15" s="31"/>
-      <c r="Q15" s="31"/>
-      <c r="R15" s="31"/>
-      <c r="S15" s="31"/>
-      <c r="T15" s="31"/>
-      <c r="U15" s="31"/>
-      <c r="V15" s="32"/>
-      <c r="W15" s="32"/>
-      <c r="X15" s="32"/>
-      <c r="Y15" s="32"/>
-      <c r="Z15" s="32"/>
-      <c r="AA15" s="32"/>
-      <c r="AB15" s="32"/>
+      <c r="B15" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="28"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+      <c r="I15" s="31"/>
+      <c r="J15" s="31"/>
+      <c r="K15" s="31"/>
+      <c r="L15" s="31"/>
+      <c r="M15" s="31"/>
+      <c r="N15" s="31"/>
+      <c r="O15" s="31"/>
+      <c r="P15" s="32"/>
+      <c r="Q15" s="32"/>
+      <c r="R15" s="32"/>
+      <c r="S15" s="32"/>
+      <c r="T15" s="32"/>
+      <c r="U15" s="32"/>
+      <c r="V15" s="33"/>
+      <c r="W15" s="33"/>
+      <c r="X15" s="33"/>
+      <c r="Y15" s="33"/>
+      <c r="Z15" s="33"/>
+      <c r="AA15" s="33"/>
+      <c r="AB15" s="33"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="35"/>
+      <c r="B16" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="30">
@@ -3145,381 +3149,381 @@
   <dimension ref="B1:N16"/>
   <sheetFormatPr defaultColWidth="8.859375" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="16.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="7.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="10.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="16.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="7.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="16.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="12.29"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="1"/>
-      <c r="D1" s="2" t="s">
+      <c r="B1" s="2"/>
+      <c r="D1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
-      <c r="E3" s="36"/>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
-      <c r="H3" s="36"/>
-      <c r="I3" s="36"/>
-      <c r="J3" s="36"/>
-      <c r="K3" s="36"/>
-      <c r="L3" s="36"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="37"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="37"/>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="37"/>
+      <c r="L3" s="37"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="39" t="s">
         <v>126</v>
       </c>
-      <c r="D4" s="39" t="s">
+      <c r="D4" s="40" t="s">
         <v>127</v>
       </c>
-      <c r="E4" s="40" t="s">
+      <c r="E4" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="F4" s="40"/>
-      <c r="G4" s="40"/>
-      <c r="H4" s="40"/>
-      <c r="I4" s="40"/>
-      <c r="J4" s="40"/>
-      <c r="K4" s="40" t="s">
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
+      <c r="J4" s="41"/>
+      <c r="K4" s="41" t="s">
         <v>129</v>
       </c>
-      <c r="L4" s="40"/>
+      <c r="L4" s="41"/>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="37"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="G5" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="I5" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41" t="s">
+      <c r="B5" s="38"/>
+      <c r="C5" s="39"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42" t="s">
         <v>130</v>
       </c>
-      <c r="L5" s="41" t="s">
+      <c r="L5" s="42" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="40" t="n">
+      <c r="B6" s="41" t="n">
         <v>9</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="43" t="s">
         <v>132</v>
       </c>
-      <c r="D6" s="43" t="s">
+      <c r="D6" s="44" t="s">
         <v>121</v>
       </c>
-      <c r="E6" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="G6" s="44" t="s">
+      <c r="E6" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="F6" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="H6" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="J6" s="44"/>
-      <c r="K6" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="L6" s="40" t="s">
+      <c r="H6" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="I6" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="J6" s="45"/>
+      <c r="K6" s="45" t="s">
+        <v>27</v>
+      </c>
+      <c r="L6" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="40" t="n">
+      <c r="B7" s="41" t="n">
         <v>10</v>
       </c>
-      <c r="C7" s="42"/>
-      <c r="D7" s="43" t="s">
+      <c r="C7" s="43"/>
+      <c r="D7" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="E7" s="40" t="n">
+      <c r="E7" s="41" t="n">
         <v>5</v>
       </c>
-      <c r="F7" s="40" t="n">
+      <c r="F7" s="41" t="n">
         <v>6</v>
       </c>
-      <c r="G7" s="40" t="s">
+      <c r="G7" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H7" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="J7" s="40"/>
-      <c r="K7" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="40" t="s">
+      <c r="H7" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="I7" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="41"/>
+      <c r="K7" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="L7" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="40" t="n">
+      <c r="B8" s="41" t="n">
         <v>11</v>
       </c>
-      <c r="C8" s="42"/>
-      <c r="D8" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="G8" s="40" t="s">
+      <c r="C8" s="43"/>
+      <c r="D8" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="F8" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="G8" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H8" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="I8" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="40" t="s">
+      <c r="H8" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="41"/>
+      <c r="K8" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="40" t="n">
+      <c r="B9" s="41" t="n">
         <v>12</v>
       </c>
-      <c r="C9" s="42"/>
-      <c r="D9" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="40" t="s">
+      <c r="C9" s="43"/>
+      <c r="D9" s="46" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="H9" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="J9" s="40"/>
-      <c r="K9" s="40" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" s="40" t="s">
+      <c r="H9" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="I9" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="41"/>
+      <c r="K9" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="L9" s="41" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="41" t="n">
+      <c r="B10" s="42" t="n">
         <v>13</v>
       </c>
-      <c r="C10" s="42"/>
-      <c r="D10" s="46" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="41" t="s">
+      <c r="C10" s="43"/>
+      <c r="D10" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="F10" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="H10" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" s="41"/>
-      <c r="K10" s="41" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="41" t="s">
+      <c r="H10" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="I10" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="42"/>
+      <c r="K10" s="42" t="s">
+        <v>27</v>
+      </c>
+      <c r="L10" s="42" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="47"/>
-      <c r="C11" s="47"/>
-      <c r="D11" s="47"/>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="47"/>
+      <c r="B11" s="48"/>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
+      <c r="E11" s="48"/>
+      <c r="F11" s="48"/>
+      <c r="G11" s="48"/>
+      <c r="H11" s="48"/>
+      <c r="I11" s="48"/>
+      <c r="J11" s="48"/>
+      <c r="K11" s="48"/>
+      <c r="L11" s="48"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="47" t="s">
+      <c r="B12" s="48" t="s">
         <v>134</v>
       </c>
-      <c r="K12" s="48"/>
+      <c r="K12" s="49"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="49" t="s">
+      <c r="B13" s="50" t="s">
         <v>135</v>
       </c>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="50" t="s">
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="51" t="s">
         <v>136</v>
       </c>
-      <c r="G13" s="50"/>
-      <c r="H13" s="51" t="s">
+      <c r="G13" s="51"/>
+      <c r="H13" s="52" t="s">
         <v>137</v>
       </c>
-      <c r="I13" s="51"/>
-      <c r="J13" s="51"/>
-      <c r="K13" s="51"/>
-      <c r="L13" s="51"/>
-      <c r="M13" s="52" t="s">
+      <c r="I13" s="52"/>
+      <c r="J13" s="52"/>
+      <c r="K13" s="52"/>
+      <c r="L13" s="52"/>
+      <c r="M13" s="53" t="s">
         <v>138</v>
       </c>
-      <c r="N13" s="52"/>
+      <c r="N13" s="53"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="53" t="s">
+      <c r="B14" s="54" t="s">
         <v>139</v>
       </c>
-      <c r="C14" s="54" t="s">
+      <c r="C14" s="55" t="s">
         <v>140</v>
       </c>
-      <c r="D14" s="54" t="s">
+      <c r="D14" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="E14" s="55" t="s">
+      <c r="E14" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="F14" s="56" t="s">
+      <c r="F14" s="57" t="s">
         <v>143</v>
       </c>
-      <c r="G14" s="57" t="s">
+      <c r="G14" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="H14" s="58" t="s">
+      <c r="H14" s="59" t="s">
         <v>145</v>
       </c>
-      <c r="I14" s="54" t="s">
+      <c r="I14" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="J14" s="54" t="s">
+      <c r="J14" s="55" t="s">
         <v>140</v>
       </c>
-      <c r="K14" s="59" t="s">
+      <c r="K14" s="60" t="s">
         <v>146</v>
       </c>
-      <c r="L14" s="60" t="s">
+      <c r="L14" s="61" t="s">
         <v>147</v>
       </c>
-      <c r="M14" s="61" t="s">
+      <c r="M14" s="62" t="s">
         <v>148</v>
       </c>
-      <c r="N14" s="62" t="s">
+      <c r="N14" s="63" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="53"/>
-      <c r="C15" s="54"/>
-      <c r="D15" s="54"/>
-      <c r="E15" s="55"/>
-      <c r="F15" s="56"/>
-      <c r="G15" s="57"/>
-      <c r="H15" s="58"/>
-      <c r="I15" s="54"/>
-      <c r="J15" s="54"/>
-      <c r="K15" s="59"/>
-      <c r="L15" s="60"/>
-      <c r="M15" s="61"/>
-      <c r="N15" s="62"/>
+      <c r="B15" s="54"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="56"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="58"/>
+      <c r="H15" s="59"/>
+      <c r="I15" s="55"/>
+      <c r="J15" s="55"/>
+      <c r="K15" s="60"/>
+      <c r="L15" s="61"/>
+      <c r="M15" s="62"/>
+      <c r="N15" s="63"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="7" t="n">
+      <c r="B16" s="8" t="n">
         <f aca="false">SUM(C16:D16)</f>
         <v>0</v>
       </c>
-      <c r="C16" s="63" t="n">
+      <c r="C16" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="D16" s="63" t="n">
+      <c r="D16" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="64"/>
-      <c r="F16" s="65"/>
-      <c r="G16" s="66" t="s">
+      <c r="E16" s="65"/>
+      <c r="F16" s="66"/>
+      <c r="G16" s="67" t="s">
         <v>150</v>
       </c>
-      <c r="H16" s="67" t="s">
+      <c r="H16" s="68" t="s">
         <v>150</v>
       </c>
-      <c r="I16" s="7" t="n">
+      <c r="I16" s="8" t="n">
         <f aca="false">SUM(J16:K16)</f>
         <v>0</v>
       </c>
-      <c r="J16" s="63" t="n">
+      <c r="J16" s="64" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="68" t="n">
+      <c r="K16" s="69" t="n">
         <v>0</v>
       </c>
-      <c r="L16" s="69"/>
-      <c r="M16" s="70" t="s">
+      <c r="L16" s="70"/>
+      <c r="M16" s="71" t="s">
         <v>150</v>
       </c>
-      <c r="N16" s="71" t="n">
+      <c r="N16" s="72" t="n">
         <f aca="false">C16</f>
         <v>0</v>
       </c>

</xml_diff>